<commit_message>
Ajout des statistiques & ameliorations dess reductions
</commit_message>
<xml_diff>
--- a/ExcelFiles/Clients.xlsx
+++ b/ExcelFiles/Clients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,14 +497,72 @@
           <t>bankole</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>204605198</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>1231231231231</t>
+      <c r="C4" t="n">
+        <v>204605198</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1231231231231</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C008</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>198505075</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bg02145LMPO1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C016</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ZOUNOU</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>198815554</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>klji1025410</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C019</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KOKOU</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>015454801</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>15451dlss</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FacturaPy fin sans interface graphique
</commit_message>
<xml_diff>
--- a/ExcelFiles/Clients.xlsx
+++ b/ExcelFiles/Clients.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,14 +555,54 @@
           <t>KOKOU</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>015454801</t>
-        </is>
+      <c r="C7" t="n">
+        <v>15454801</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>15451dlss</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C0078</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mael</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>40464164</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C079</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mael</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>40454545</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1231231231231</t>
         </is>
       </c>
     </row>

</xml_diff>